<commit_message>
updated on 1 SEP
</commit_message>
<xml_diff>
--- a/CAP776 (PYTHON).xlsx
+++ b/CAP776 (PYTHON).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\palak\Downloads\776(clone)\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87CBFFE-6098-49E3-89BB-70DF1752347E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5088BE-7B5E-43C7-B38C-718E10B48D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{327CE7B2-1886-45B8-951C-28CB36CE6AAF}"/>
   </bookViews>
@@ -434,22 +434,22 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -785,39 +785,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
       <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="26">
         <v>12617802</v>
       </c>
-      <c r="G2" s="21"/>
+      <c r="G2" s="26"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -830,18 +830,18 @@
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="21"/>
+      <c r="G3" s="26"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -851,22 +851,22 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
     </row>
     <row r="5" spans="1:14" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -913,7 +913,7 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="23">
+      <c r="A6" s="20">
         <v>46246</v>
       </c>
       <c r="B6" s="9">
@@ -957,7 +957,7 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="23">
+      <c r="A7" s="20">
         <v>46247</v>
       </c>
       <c r="B7" s="9">
@@ -1001,7 +1001,7 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="23">
+      <c r="A8" s="20">
         <v>46248</v>
       </c>
       <c r="B8" s="9">
@@ -1045,7 +1045,7 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="23">
+      <c r="A9" s="20">
         <v>46249</v>
       </c>
       <c r="B9" s="9">
@@ -1089,7 +1089,7 @@
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="23">
+      <c r="A10" s="20">
         <v>46250</v>
       </c>
       <c r="B10" s="9">
@@ -1133,7 +1133,7 @@
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="23">
+      <c r="A11" s="20">
         <v>46251</v>
       </c>
       <c r="B11" s="10">
@@ -1177,7 +1177,7 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="23">
+      <c r="A12" s="20">
         <v>46252</v>
       </c>
       <c r="B12" s="10">
@@ -1221,7 +1221,7 @@
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="23">
+      <c r="A13" s="20">
         <v>46253</v>
       </c>
       <c r="B13" s="10">
@@ -1265,7 +1265,7 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="23">
+      <c r="A14" s="20">
         <v>46254</v>
       </c>
       <c r="B14" s="10">
@@ -1309,7 +1309,7 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="23">
+      <c r="A15" s="20">
         <v>46255</v>
       </c>
       <c r="B15" s="10">
@@ -1353,7 +1353,7 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="23">
+      <c r="A16" s="20">
         <v>46256</v>
       </c>
       <c r="B16" s="10">
@@ -1397,7 +1397,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="23">
+      <c r="A17" s="20">
         <v>46257</v>
       </c>
       <c r="B17" s="10">
@@ -1442,7 +1442,7 @@
       <c r="O17" s="10"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="24">
+      <c r="A18" s="23">
         <v>46258</v>
       </c>
       <c r="B18" s="10">
@@ -1486,7 +1486,7 @@
       </c>
     </row>
     <row r="19" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="23">
+      <c r="A19" s="20">
         <v>46259</v>
       </c>
       <c r="B19" s="10">
@@ -1530,7 +1530,7 @@
       </c>
     </row>
     <row r="20" spans="1:15" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="23">
+      <c r="A20" s="20">
         <v>46260</v>
       </c>
       <c r="B20" s="12">
@@ -1574,7 +1574,7 @@
       </c>
     </row>
     <row r="21" spans="1:15" ht="13.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="23">
+      <c r="A21" s="20">
         <v>46261</v>
       </c>
       <c r="B21" s="14">
@@ -1618,7 +1618,7 @@
       </c>
     </row>
     <row r="22" spans="1:15" ht="13.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="25">
+      <c r="A22" s="21">
         <v>46262</v>
       </c>
       <c r="B22" s="15">
@@ -1662,7 +1662,7 @@
       </c>
     </row>
     <row r="23" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="25">
+      <c r="A23" s="21">
         <v>46263</v>
       </c>
       <c r="B23" s="15">
@@ -1706,7 +1706,7 @@
       </c>
     </row>
     <row r="24" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="25">
+      <c r="A24" s="21">
         <v>46264</v>
       </c>
       <c r="B24" s="15">
@@ -1750,7 +1750,7 @@
       </c>
     </row>
     <row r="25" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="25">
+      <c r="A25" s="21">
         <v>46265</v>
       </c>
       <c r="B25" s="15">
@@ -1794,7 +1794,7 @@
       </c>
     </row>
     <row r="26" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="25">
+      <c r="A26" s="21">
         <v>46266</v>
       </c>
       <c r="B26" s="15">
@@ -1838,7 +1838,7 @@
       </c>
     </row>
     <row r="27" spans="1:15" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="25">
+      <c r="A27" s="21">
         <v>46267</v>
       </c>
       <c r="B27" s="16">
@@ -1882,7 +1882,7 @@
       </c>
     </row>
     <row r="28" spans="1:15" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="25">
+      <c r="A28" s="21">
         <v>46268</v>
       </c>
       <c r="B28" s="16">
@@ -1926,7 +1926,7 @@
       </c>
     </row>
     <row r="29" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="25">
+      <c r="A29" s="21">
         <v>46269</v>
       </c>
       <c r="B29" s="16">
@@ -1970,7 +1970,7 @@
       </c>
     </row>
     <row r="30" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="25">
+      <c r="A30" s="21">
         <v>46270</v>
       </c>
       <c r="B30" s="16">
@@ -2014,7 +2014,7 @@
       </c>
     </row>
     <row r="31" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="26">
+      <c r="A31" s="22">
         <v>46271</v>
       </c>
       <c r="B31" s="13">
@@ -2058,7 +2058,7 @@
       </c>
     </row>
     <row r="32" spans="1:15" ht="19.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="26">
+      <c r="A32" s="22">
         <v>46272</v>
       </c>
       <c r="B32" s="13">
@@ -2102,7 +2102,7 @@
       </c>
     </row>
     <row r="33" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="26">
+      <c r="A33" s="22">
         <v>46273</v>
       </c>
       <c r="B33" s="13">
@@ -2141,12 +2141,12 @@
       <c r="M33" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N33" s="22" t="s">
+      <c r="N33" s="19" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="26">
+      <c r="A34" s="22">
         <v>46274</v>
       </c>
       <c r="B34" s="13">
@@ -2185,12 +2185,12 @@
       <c r="M34" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="N34" s="22" t="s">
+      <c r="N34" s="19" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="26">
+      <c r="A35" s="22">
         <v>46275</v>
       </c>
       <c r="B35" s="13">
@@ -2229,12 +2229,12 @@
       <c r="M35" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N35" s="22" t="s">
+      <c r="N35" s="19" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="26">
+      <c r="A36" s="22">
         <v>46276</v>
       </c>
       <c r="B36" s="13">
@@ -2273,7 +2273,7 @@
       <c r="M36" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="N36" s="22" t="s">
+      <c r="N36" s="19" t="s">
         <v>70</v>
       </c>
     </row>
@@ -9655,5 +9655,6 @@
     <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>